<commit_message>
Generating updated summaries for manuscript
</commit_message>
<xml_diff>
--- a/logs/data_processing.xlsx
+++ b/logs/data_processing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryanm\Documents\PhD\GitHub\attrisk\logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD58D184-8975-4923-8111-A7ADE8796483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9FCCA8-14E9-4319-87C8-8274F7B27023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32805" yWindow="1485" windowWidth="20025" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="prepare_data" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="156">
   <si>
     <t>stage</t>
   </si>
@@ -437,9 +437,6 @@
     <t>ipd trials provided AgD so are included at both levels of risk prediction model framework</t>
   </si>
   <si>
-    <t>None/Unknown; &lt;=80; &gt;80</t>
-  </si>
-  <si>
     <t>None/Unknown; 18; &gt;18</t>
   </si>
   <si>
@@ -486,6 +483,18 @@
   </si>
   <si>
     <t>Reference captures 3 trials designated as "Not applicable" in design features</t>
+  </si>
+  <si>
+    <t>None/Unknown; 80; &gt;80</t>
+  </si>
+  <si>
+    <t>removed ipd trials with less than 10 events per non-experimental arm</t>
+  </si>
+  <si>
+    <t>model would not fit if these were included in relevant trials</t>
+  </si>
+  <si>
+    <t>the total is 342 and 76 have ipd; agd for all 342 trials</t>
   </si>
 </sst>
 </file>
@@ -809,7 +818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -885,6 +894,29 @@
       </c>
       <c r="F3" s="1">
         <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D4" s="1">
+        <v>342</v>
+      </c>
+      <c r="E4" s="1">
+        <v>342</v>
+      </c>
+      <c r="F4" s="1">
+        <v>76</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -3351,7 +3383,7 @@
         <v>91</v>
       </c>
       <c r="D1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E1" t="s">
         <v>117</v>
@@ -3374,13 +3406,13 @@
         <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E2" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="F2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3394,13 +3426,13 @@
         <v>97</v>
       </c>
       <c r="D3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -3414,13 +3446,13 @@
         <v>101</v>
       </c>
       <c r="D4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -3434,13 +3466,13 @@
         <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -3454,13 +3486,13 @@
         <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -3474,13 +3506,13 @@
         <v>106</v>
       </c>
       <c r="D7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E7" t="s">
         <v>107</v>
       </c>
       <c r="F7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -3494,13 +3526,13 @@
         <v>109</v>
       </c>
       <c r="D8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -3514,13 +3546,13 @@
         <v>111</v>
       </c>
       <c r="D9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -3534,16 +3566,16 @@
         <v>112</v>
       </c>
       <c r="D10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F10" t="s">
+        <v>150</v>
+      </c>
+      <c r="G10" t="s">
         <v>151</v>
-      </c>
-      <c r="G10" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -3557,13 +3589,13 @@
         <v>113</v>
       </c>
       <c r="D11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -3577,13 +3609,13 @@
         <v>114</v>
       </c>
       <c r="D12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -3597,10 +3629,10 @@
         <v>115</v>
       </c>
       <c r="D13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F13" t="s">
         <v>120</v>
@@ -3617,10 +3649,10 @@
         <v>116</v>
       </c>
       <c r="D14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F14" t="s">
         <v>120</v>
@@ -3637,7 +3669,7 @@
         <v>128</v>
       </c>
       <c r="D15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E15" t="s">
         <v>134</v>
@@ -3657,7 +3689,7 @@
         <v>129</v>
       </c>
       <c r="D16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E16" t="s">
         <v>134</v>
@@ -3677,7 +3709,7 @@
         <v>130</v>
       </c>
       <c r="D17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E17" t="s">
         <v>134</v>
@@ -3697,7 +3729,7 @@
         <v>131</v>
       </c>
       <c r="D18" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E18" t="s">
         <v>134</v>
@@ -3717,7 +3749,7 @@
         <v>132</v>
       </c>
       <c r="D19" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E19" t="s">
         <v>134</v>
@@ -3737,7 +3769,7 @@
         <v>133</v>
       </c>
       <c r="D20" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E20" t="s">
         <v>134</v>

</xml_diff>

<commit_message>
Additional manuscript summary and output tidying updates
</commit_message>
<xml_diff>
--- a/logs/data_processing.xlsx
+++ b/logs/data_processing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryanm\Documents\PhD\GitHub\attrisk\logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9FCCA8-14E9-4319-87C8-8274F7B27023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5DDC57-13AD-44B0-B6B4-E38E80F39DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32805" yWindow="1485" windowWidth="20025" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33150" yWindow="1830" windowWidth="20025" windowHeight="13590" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="prepare_data" sheetId="1" r:id="rId1"/>
@@ -467,9 +467,6 @@
     <t>0 = phase 3 or unknown; 1 = phase 4</t>
   </si>
   <si>
-    <t>2; 3; &gt;3</t>
-  </si>
-  <si>
     <t>&lt;100; 100-199; &gt;=200</t>
   </si>
   <si>
@@ -495,6 +492,9 @@
   </si>
   <si>
     <t>the total is 342 and 76 have ipd; agd for all 342 trials</t>
+  </si>
+  <si>
+    <t>2; &gt;2</t>
   </si>
 </sst>
 </file>
@@ -901,10 +901,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="D4" s="1">
         <v>342</v>
@@ -916,7 +916,7 @@
         <v>76</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -3409,10 +3409,10 @@
         <v>138</v>
       </c>
       <c r="E2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3432,7 +3432,7 @@
         <v>136</v>
       </c>
       <c r="F3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -3452,7 +3452,7 @@
         <v>140</v>
       </c>
       <c r="F4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -3472,7 +3472,7 @@
         <v>141</v>
       </c>
       <c r="F5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -3492,7 +3492,7 @@
         <v>142</v>
       </c>
       <c r="F6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -3512,7 +3512,7 @@
         <v>107</v>
       </c>
       <c r="F7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -3532,7 +3532,7 @@
         <v>143</v>
       </c>
       <c r="F8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -3552,7 +3552,7 @@
         <v>144</v>
       </c>
       <c r="F9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -3572,10 +3572,10 @@
         <v>145</v>
       </c>
       <c r="F10" t="s">
+        <v>149</v>
+      </c>
+      <c r="G10" t="s">
         <v>150</v>
-      </c>
-      <c r="G10" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -3592,10 +3592,10 @@
         <v>138</v>
       </c>
       <c r="E11" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="F11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -3612,10 +3612,10 @@
         <v>138</v>
       </c>
       <c r="E12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F12" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -3632,7 +3632,7 @@
         <v>139</v>
       </c>
       <c r="E13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F13" t="s">
         <v>120</v>
@@ -3652,7 +3652,7 @@
         <v>138</v>
       </c>
       <c r="E14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F14" t="s">
         <v>120</v>

</xml_diff>